<commit_message>
Se agregó la R7 para limitación de la corriente de base de Q2.
</commit_message>
<xml_diff>
--- a/Bill of Materials Placa Corte TX.xlsx
+++ b/Bill of Materials Placa Corte TX.xlsx
@@ -72,9 +72,6 @@
     <t>Q2</t>
   </si>
   <si>
-    <t>R1, R5</t>
-  </si>
-  <si>
     <t>R2</t>
   </si>
   <si>
@@ -172,6 +169,9 @@
   </si>
   <si>
     <t>Conector macho de inserción (THT), 1 fila de 4 pines, paso estándar de 2.54 mm (0.1")</t>
+  </si>
+  <si>
+    <t>R1, R5, R7</t>
   </si>
 </sst>
 </file>
@@ -1127,10 +1127,10 @@
         <v>60020011</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1144,10 +1144,10 @@
         <v>60040119</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1161,10 +1161,10 @@
         <v>60041001</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1178,10 +1178,10 @@
         <v>60002025</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1195,10 +1195,10 @@
         <v>60000002</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1215,7 +1215,7 @@
         <v>4</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1229,10 +1229,10 @@
         <v>60090004</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1246,10 +1246,10 @@
         <v>60053001</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1263,32 +1263,32 @@
         <v>60053000</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B12" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="3">
         <v>60012080</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B13" s="3">
         <v>1</v>
@@ -1297,15 +1297,15 @@
         <v>60012027</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14" s="3">
         <v>1</v>
@@ -1314,15 +1314,15 @@
         <v>60012065</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B15" s="3">
         <v>1</v>
@@ -1331,15 +1331,15 @@
         <v>60012012</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B16" s="3">
         <v>1</v>
@@ -1348,10 +1348,10 @@
         <v>60012071</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1365,10 +1365,10 @@
         <v>60069210</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>